<commit_message>
Time Travel Rev 6: Serp aus dem ganzen Plan, Serie REWIND, Datenschutz auf 23.10.
- W5–W32: Serp aus allen Aufgaben ab 13.10. geschnitten (an Ort und Stelle,
  keine Aufgabe eingefügt oder verschoben), Stich-Deckel 28.000
- Kalkulation 59,90 €/Paar, Prüfplan, Urteil, Countdown-Liste und Analysen nachgeführt
- Serie REWIND: 20 Stunt-Videos mit Dreh-, Schnitt-, Post- und Making-of-Aufgaben
  (extra.json aus build/rewind_data.py), Feld „Codewort“ am 11.11.
- Datenschutz-Absätze für Tally und „Bring 3“ auf Fr 23.10. verschoben,
  Freischalten erst danach
- Build-Quellen (build/) jetzt versioniert
- Docket veröffentlicht als Version 16

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TWy6p8o9SQF8kE6aYDsvrE
</commit_message>
<xml_diff>
--- a/novalife/time-travel/rev6/2026-10-11_time-travel-tracking.xlsx
+++ b/novalife/time-travel/rev6/2026-10-11_time-travel-tracking.xlsx
@@ -780,7 +780,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Papiertest-3-Antworten P1–P10 mit Zähler für die Serp-Regel.</t>
+          <t>Papiertest-3-Antworten P1–P10 (Serp seit 11.10. gestrichen).</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Codes P1–P10 mit Segment. Regel Serp: 0 Sowjet/Wappen-Nennungen → Rot bleibt · 1 → du entscheidest · ≥ 2 → grau · ≥ 4 → Serp nicht in dieser Größe.</t>
+          <t>Codes P1–P10 mit Segment. Die Serp-Regel ist erledigt, der Serp ist seit 11.10. gestrichen. Die Antworten zählen weiter für Zielgruppe und Preis.</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7100,7 +7100,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Serp-Farbe nach Testregel, B2-Kante, V1 Nummer, V5 Patch, V6 Karte, Taschenklappe, Nackenlabel (mit Novalife-Adresse), „goldene Nähte“, Namen nach außen</t>
+          <t>Serp-Farbe nach Testregel (entfällt, siehe 11.10.), B2-Kante, V1 Nummer, V5 Patch, V6 Karte, Taschenklappe, Nackenlabel (mit Novalife-Adresse), „goldene Nähte“, Namen nach außen</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -7115,179 +7115,179 @@
           <t>So 11.10.</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Innenbein-Gradierung +1,0 oder +1,5</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>kein eigener Rat, mir fehlen Daten. Die Spec steht auf +1,0; ohne Grund für +1,5 bleibt es dabei</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Entschieden: Serp gestrichen · Patch D wird die hintere Gürtelschlaufe (nur seitlich genäht und genietet) · Größe B, 76 × 67 mm, 3–5 mm Spiel</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>erledigt</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Do 15.10.</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Wie viel Familie in den Content; Teppich für den Shoot leihen</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>über Gegenstände, nicht über Länder</t>
+          <t>So 11.10.</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Innenbein-Gradierung +1,0 oder +1,5</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>kein eigener Rat, mir fehlen Daten. Die Spec steht auf +1,0; ohne Grund für +1,5 bleibt es dabei</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>So 18.10.</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Pixel-Spiel</t>
+          <t>Do 15.10.</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Wie viel Familie in den Content; Teppich für den Shoot leihen</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>streichen, Scroll-Story B</t>
+          <t>über Gegenstände, nicht über Länder</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Di 20.10.</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Baum-Referenz: eigene oder fremde Vorlage?</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>fremd → Claude zeichnet eine eigene Fassung vor dem 28.10.</t>
+          <t>So 18.10.</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Pixel-Spiel</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>streichen, Scroll-Story B</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Di 27.10.</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>DAP oder DDP</t>
+          <t>Di 20.10.</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Patch D: mittig auf der hinteren Mittelnaht oder rechts daneben; „NL“ auf dem Patch</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>DAP, damit die Steuer nicht schon in der Restzahlung steckt</t>
+          <t>mittig, wenn die Fabrik Nieten über der Mittelnaht bestätigt; NL wie auf dem Foto</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Sa 07.11.</t>
+          <t>Di 20.10.</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Sprache der Hooks und damit das Liefergebiet; Bildregel „keine Seitenansicht links“</t>
+          <t>Baum-Referenz: eigene oder fremde Vorlage?</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Test entscheidet; deutsch → nur Versand nach DE bis zum Drop; Bildregel halten</t>
+          <t>fremd → Claude zeichnet eine eigene Fassung vor dem 28.10.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>So 29.11.</t>
+          <t>ab So 01.11.</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>„Platz in der ersten Stunde sichern“ A (10 €) oder B (kostenlos)</t>
+          <t>IHK-Gründungsberatung (angefragt am 13.10.), danach Gewerbe anmelden</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>B, A nur bei Liste &lt; 170 und grünem Recht</t>
+          <t>anmelden vor der ersten Vorbestellung und bevor Rechnungen auf deinen Namen laufen; online geht es in 20 Minuten</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Fr 11.12.</t>
+          <t>Di 27.10.</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Creator-Abmachung 1 Clip + 1 Story</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>DAP oder DDP</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>DAP, damit die Steuer nicht schon in der Restzahlung steckt</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Mo 14.12.</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>Liefertext</t>
+          <t>Sa 07.11.</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Sprache der Hooks und damit das Liefergebiet; Bildregel „keine Seitenansicht links“</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>„Lieferung bis spätestens 30.04.2027, geplant Anfang April“, überall derselbe Satz</t>
+          <t>Test entscheidet; deutsch → nur Versand nach DE bis zum Drop; Bildregel halten</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Di 15.12.</t>
+          <t>So 29.11.</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Geld-zurück-Regel, Vorbestellgeld bis 01.02. unangetastet</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>„Platz in der ersten Stunde sichern“ A (10 €) oder B (kostenlos)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>B, A nur bei Liste &lt; 170 und grünem Recht</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Sa 19.12.</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Stufe 2 zu 169 € statt Kontingent 45; Nummern 001–035 · 036–060 · 061–065 · 066–067 · Rest</t>
+          <t>Fr 11.12.</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Creator-Abmachung 1 Clip + 1 Story</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -7299,83 +7299,134 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Do 31.12.</t>
+          <t>Mo 14.12.</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Brücke 1.500 € in der Familie</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>anfragen, nur als Versicherung</t>
+          <t>Liefertext</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>„Lieferung bis spätestens 30.04.2027, geplant Anfang April“, überall derselbe Satz</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>So 24.01.</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Mess-Abend 2b (Mi 27.01.)</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>ja, wenn am 13.01. &lt; 60 Reservierungen + Zusagen oder Vorbestellungen unter Soll</t>
+          <t>Di 15.12.</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Geld-zurück-Regel, Vorbestellgeld bis 01.02. unangetastet</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>ja</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Mo 01.02.</t>
+          <t>Sa 19.12.</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Mengenformel 100/75; Notfall-Option Zipper bei 7–9</t>
+          <t>Stufe 2 zu 169 € statt Kontingent 45; Nummern 001–035 · 036–060 · 061–065 · 066–067 · Rest</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>ja / bereithalten</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Fr 05.03.</t>
+          <t>Do 31.12.</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Drop-Abend Sa 24.04.; Countdown-Stand</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>ja nur, wenn Packen Tag 2 an die Helfer geht oder auf So 25.04. rückt / nur unter ~146 €</t>
+          <t>Brücke 1.500 € in der Familie</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>anfragen, nur als Versicherung</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
+          <t>So 24.01.</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Mess-Abend 2b (Mi 27.01.)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>ja, wenn am 13.01. &lt; 60 Reservierungen + Zusagen oder Vorbestellungen unter Soll</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Mo 01.02.</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Mengenformel 100/75; Notfall-Option Zipper bei 7–9</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>ja / bereithalten</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Fr 05.03.</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Drop-Abend Sa 24.04.; Countdown-Stand</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>ja nur, wenn Packen Tag 2 an die Helfer geht oder auf So 25.04. rückt / nur unter ~146 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
           <t>nach dem Drop</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Marke „Novalife“ anmelden; W28 in den Größenlauf</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Markenrecherche vom 16.10. und Nachfrage „kleiner als W30“ auswerten, erst dann rechnen</t>
         </is>
@@ -8497,7 +8548,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Ampel rot: Gegenrechnung, Optionen V4b, kleiner Serp, 75 Stück</t>
+          <t>Ampel rot: Gegenrechnung, Optionen V4b, 75 Stück</t>
         </is>
       </c>
     </row>
@@ -8553,7 +8604,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Farbe B/B2, Namen, Sprache final, Bildregel „keine Seitenansicht links“, Liefergebiet</t>
+          <t>Farbe B2-Kante, Namen, Sprache final, Liefergebiet</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -8563,7 +8614,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Ohne Daten gilt der Rat: graue Schneide, weiße Kante, Wortliste, EN-Hook mit DE-Zeile, Bildregel bleibt</t>
+          <t>Ohne Daten gilt der Rat: weiße Kante, Wortliste, EN-Hook mit DE-Zeile</t>
         </is>
       </c>
     </row>
@@ -8595,9 +8646,9 @@
           <t>Di 10.11.</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>Stiche ≤ 33.000</t>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Stiche ≤ 28.000 (seit 11.10. ohne Serp, vorher 33.000)</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Time Travel Rev 6: Drop verschoben auf Do 24.06.2027 (Abitur)
- Bis W18 unverändert, Aufholwochen W19 und W22, Abi-Pause W28–W34 (22.03.–09.05.)
- Alte W19–W32 auf W20–W41 umgerechnet, alle Daten im Text mitgezogen,
  Kalenderfeste Termine (24.02., Ramadan, Ostern, Sperrwoche) bleiben echt
- Fabrik: Ware fertig bis Fr 14.05. (vor dem Opferfest), Restzahlung Fr 21.05.
- Autopilot-Posts für die Pause, Liefersatz „bis spätestens 30.06.2027, geplant Anfang Juni“
- Countdown, Phasen, Cockpit (41 Wochen), Kalkulation, Zeitachse, Strategie,
  Analysen und REWIND-Termine nachgeführt, Entscheidung 13.10. im Urteil
- Docket veröffentlicht als Version 17

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TWy6p8o9SQF8kE6aYDsvrE
</commit_message>
<xml_diff>
--- a/novalife/time-travel/rev6/2026-10-11_time-travel-tracking.xlsx
+++ b/novalife/time-travel/rev6/2026-10-11_time-travel-tracking.xlsx
@@ -1951,7 +1951,7 @@
       </c>
       <c r="N3" s="9" t="inlineStr">
         <is>
-          <t>Story 17.–21.04.</t>
+          <t>Story 19.–23.06.</t>
         </is>
       </c>
       <c r="O3" s="9" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2939,14 +2939,14 @@
         </is>
       </c>
       <c r="C19" s="11" t="n">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>520</v>
+        <v>450</v>
       </c>
       <c r="E19" s="12" t="n"/>
       <c r="F19" s="11" t="n">
-        <v>3750</v>
+        <v>3000</v>
       </c>
       <c r="G19" s="12" t="n"/>
       <c r="H19">
@@ -2955,10 +2955,10 @@
       </c>
       <c r="J19" s="12" t="n"/>
       <c r="K19" s="11" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="L19" s="11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M19" s="12" t="n"/>
       <c r="N19">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>So 24.01.: eigene Kaufquote (Vorbestellungen ÷ Liste 13.01.) · Mess-Abend 2b · Patches bei der Fabrik</t>
+          <t>Aufholwoche: keine neuen Gates</t>
         </is>
       </c>
     </row>
@@ -2981,14 +2981,14 @@
         </is>
       </c>
       <c r="C20" s="11" t="n">
-        <v>1500</v>
+        <v>1250</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>600</v>
+        <v>520</v>
       </c>
       <c r="E20" s="12" t="n"/>
       <c r="F20" s="11" t="n">
-        <v>4500</v>
+        <v>3750</v>
       </c>
       <c r="G20" s="12" t="n"/>
       <c r="H20">
@@ -2997,10 +2997,10 @@
       </c>
       <c r="J20" s="12" t="n"/>
       <c r="K20" s="11" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L20" s="11" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="M20" s="12" t="n"/>
       <c r="N20">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Sonntags-Check: Warteliste, Follower, Zusagen bzw. Vorbestellungen gegen das Soll, dazu Kassen-Ampel und Anmeldungen je 1.000 Views (Abschnitt Gates).</t>
+          <t>So 31.01.: eigene Kaufquote (Vorbestellungen ÷ Liste 13.01.) · Mess-Abend 2b · Patches bei der Fabrik</t>
         </is>
       </c>
     </row>
@@ -3023,14 +3023,14 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>1700</v>
+        <v>1500</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>660</v>
+        <v>600</v>
       </c>
       <c r="E21" s="12" t="n"/>
       <c r="F21" s="11" t="n">
-        <v>5100</v>
+        <v>4500</v>
       </c>
       <c r="G21" s="12" t="n"/>
       <c r="H21">
@@ -3039,10 +3039,10 @@
       </c>
       <c r="J21" s="12" t="n"/>
       <c r="K21" s="11" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L21" s="11" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M21" s="12" t="n"/>
       <c r="N21">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>Mo 01.02.: Schwelle 1 + Mengenformel (ausgezahlt am 31.01. + 6 × Wochenrate W19–W20) · Fr 05.02.: Spiel · So 07.02.: PO bestätigt, Anzahlung bezahlt</t>
+          <t>Sonntags-Check: Warteliste, Follower, Zusagen bzw. Vorbestellungen gegen das Soll, dazu Kassen-Ampel und Anmeldungen je 1.000 Views (Abschnitt Gates).</t>
         </is>
       </c>
     </row>
@@ -3065,14 +3065,14 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>1900</v>
+        <v>1500</v>
       </c>
       <c r="D22" s="11" t="n">
-        <v>720</v>
+        <v>600</v>
       </c>
       <c r="E22" s="12" t="n"/>
       <c r="F22" s="11" t="n">
-        <v>5700</v>
+        <v>4500</v>
       </c>
       <c r="G22" s="12" t="n"/>
       <c r="H22">
@@ -3081,10 +3081,10 @@
       </c>
       <c r="J22" s="12" t="n"/>
       <c r="K22" s="11" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L22" s="11" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="M22" s="12" t="n"/>
       <c r="N22">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>So 14.02.: Stoff da (reserviert seit 06.01.)</t>
+          <t>Aufholwoche: keine neuen Gates</t>
         </is>
       </c>
     </row>
@@ -3107,14 +3107,14 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>2150</v>
+        <v>1700</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>790</v>
+        <v>660</v>
       </c>
       <c r="E23" s="12" t="n"/>
       <c r="F23" s="11" t="n">
-        <v>6450</v>
+        <v>5100</v>
       </c>
       <c r="G23" s="12" t="n"/>
       <c r="H23">
@@ -3123,10 +3123,10 @@
       </c>
       <c r="J23" s="12" t="n"/>
       <c r="K23" s="11" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="L23" s="11" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="M23" s="12" t="n"/>
       <c r="N23">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>So 21.02.: Inline-Fotos 1</t>
+          <t>Mo 15.02.: Schwelle 1 + Mengenformel (ausgezahlt am 07.02. + 6 × Wochenrate W19–W20) · Fr 19.02.: Spiel · So 21.02.: PO bestätigt, Anzahlung bezahlt</t>
         </is>
       </c>
     </row>
@@ -3149,14 +3149,14 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>2400</v>
+        <v>1900</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>850</v>
+        <v>720</v>
       </c>
       <c r="E24" s="12" t="n"/>
       <c r="F24" s="11" t="n">
-        <v>7200</v>
+        <v>5700</v>
       </c>
       <c r="G24" s="12" t="n"/>
       <c r="H24">
@@ -3165,10 +3165,10 @@
       </c>
       <c r="J24" s="12" t="n"/>
       <c r="K24" s="11" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="L24" s="11" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M24" s="12" t="n"/>
       <c r="N24">
@@ -3177,7 +3177,7 @@
       </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>So 28.02.: ≥ 18 Vorbestellungen, Liste ≥ 850, Shopify-Email-Kontingent</t>
+          <t>So 28.02.: Stoff da (reserviert seit 06.01.)</t>
         </is>
       </c>
     </row>
@@ -3191,14 +3191,14 @@
         </is>
       </c>
       <c r="C25" s="11" t="n">
-        <v>2450</v>
+        <v>2150</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>880</v>
+        <v>790</v>
       </c>
       <c r="E25" s="12" t="n"/>
       <c r="F25" s="11" t="n">
-        <v>7350</v>
+        <v>6450</v>
       </c>
       <c r="G25" s="12" t="n"/>
       <c r="H25">
@@ -3207,10 +3207,10 @@
       </c>
       <c r="J25" s="12" t="n"/>
       <c r="K25" s="11" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="M25" s="12" t="n"/>
       <c r="N25">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>So 07.03.: Inline-Fotos 2, Steuer-Rücklage</t>
+          <t>So 07.03.: Inline-Fotos 1</t>
         </is>
       </c>
     </row>
@@ -3233,14 +3233,14 @@
         </is>
       </c>
       <c r="C26" s="11" t="n">
-        <v>2500</v>
+        <v>2400</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>910</v>
+        <v>850</v>
       </c>
       <c r="E26" s="12" t="n"/>
       <c r="F26" s="11" t="n">
-        <v>7500</v>
+        <v>7200</v>
       </c>
       <c r="G26" s="12" t="n"/>
       <c r="H26">
@@ -3249,10 +3249,10 @@
       </c>
       <c r="J26" s="12" t="n"/>
       <c r="K26" s="11" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="L26" s="11" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="M26" s="12" t="n"/>
       <c r="N26">
@@ -3261,7 +3261,7 @@
       </c>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>So 14.03.: ≥ 29 (Alarm 25) · absehbar 32 ausgezahlt bis Di 16.03. (mit der Auszahlungsdauer vom 29.12.)</t>
+          <t>So 14.03.: ≥ 18 Vorbestellungen, Liste ≥ 850, Shopify-Email-Kontingent</t>
         </is>
       </c>
     </row>
@@ -3275,14 +3275,14 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>2560</v>
+        <v>2450</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>950</v>
+        <v>880</v>
       </c>
       <c r="E27" s="12" t="n"/>
       <c r="F27" s="11" t="n">
-        <v>7680</v>
+        <v>7350</v>
       </c>
       <c r="G27" s="12" t="n"/>
       <c r="H27">
@@ -3291,10 +3291,10 @@
       </c>
       <c r="J27" s="12" t="n"/>
       <c r="K27" s="11" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="L27" s="11" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="M27" s="12" t="n"/>
       <c r="N27">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Fr 19.03.: ≥ 32 ausgezahlt bis Di 16.03. und Endkontroll-Nachweis aus der PO vollständig · So 21.03., 20:00: 35 zu 149 € voll</t>
+          <t>So 21.03.: Inline-Fotos 2, Steuer-Rücklage</t>
         </is>
       </c>
     </row>
@@ -3317,14 +3317,14 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>2620</v>
+        <v>2450</v>
       </c>
       <c r="D28" s="11" t="n">
-        <v>1050</v>
+        <v>880</v>
       </c>
       <c r="E28" s="12" t="n"/>
       <c r="F28" s="11" t="n">
-        <v>7860</v>
+        <v>7350</v>
       </c>
       <c r="G28" s="12" t="n"/>
       <c r="H28">
@@ -3333,10 +3333,10 @@
       </c>
       <c r="J28" s="12" t="n"/>
       <c r="K28" s="11" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="L28" s="11" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="M28" s="12" t="n"/>
       <c r="N28">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>Mi 24.03.: Tracking da · bei Steuer (DAP): 40 ausgezahlt (35 + Stufe 2) · So 28.03.: Ware mit Tracking, Stufe 2 ≥ 2, Kasse deckt die Steuer</t>
+          <t>Abi-Pause: keine Gates, Zahlen nur eintragen, wenn du magst</t>
         </is>
       </c>
     </row>
@@ -3359,14 +3359,14 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>2720</v>
+        <v>2450</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>1170</v>
+        <v>880</v>
       </c>
       <c r="E29" s="12" t="n"/>
       <c r="F29" s="11" t="n">
-        <v>8160</v>
+        <v>7350</v>
       </c>
       <c r="G29" s="12" t="n"/>
       <c r="H29">
@@ -3375,7 +3375,10 @@
       </c>
       <c r="J29" s="12" t="n"/>
       <c r="K29" s="11" t="n">
-        <v>43</v>
+        <v>26</v>
+      </c>
+      <c r="L29" s="11" t="n">
+        <v>21</v>
       </c>
       <c r="M29" s="12" t="n"/>
       <c r="N29">
@@ -3384,7 +3387,7 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>So 04.04.: Ware geprüft, Steuer bezahlt</t>
+          <t>Abi-Pause: keine Gates, Zahlen nur eintragen, wenn du magst</t>
         </is>
       </c>
     </row>
@@ -3398,14 +3401,14 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>2820</v>
+        <v>2450</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>1290</v>
+        <v>880</v>
       </c>
       <c r="E30" s="12" t="n"/>
       <c r="F30" s="11" t="n">
-        <v>8460</v>
+        <v>7350</v>
       </c>
       <c r="G30" s="12" t="n"/>
       <c r="H30">
@@ -3413,6 +3416,12 @@
         <v/>
       </c>
       <c r="J30" s="12" t="n"/>
+      <c r="K30" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="L30" s="11" t="n">
+        <v>21</v>
+      </c>
       <c r="M30" s="12" t="n"/>
       <c r="N30">
         <f>IF(AND(E30="",H30="",J30="",M30=""),"offen",IF(OR(AND(E30&lt;&gt;"",D30&lt;&gt;"",E30&lt;D30),AND(M30&lt;&gt;"",L30&lt;&gt;"",M30&lt;L30)),"unter Alarm",IF(OR(AND(E30&lt;&gt;"",E30&lt;C30),AND(H30&lt;&gt;"",F30&lt;&gt;"",H30&lt;F30),AND(J30&lt;&gt;"",I30&lt;&gt;"",J30&lt;I30),AND(M30&lt;&gt;"",K30&lt;&gt;"",M30&lt;K30)),"unter Soll","im Plan")))</f>
@@ -3420,7 +3429,7 @@
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Sonntags-Check: Warteliste, Follower, Zusagen bzw. Vorbestellungen gegen das Soll, dazu Kassen-Ampel und Anmeldungen je 1.000 Views (Abschnitt Gates).</t>
+          <t>Abi-Pause: keine Gates, Zahlen nur eintragen, wenn du magst</t>
         </is>
       </c>
     </row>
@@ -3434,14 +3443,14 @@
         </is>
       </c>
       <c r="C31" s="11" t="n">
-        <v>2920</v>
+        <v>2450</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>1400</v>
+        <v>880</v>
       </c>
       <c r="E31" s="12" t="n"/>
       <c r="F31" s="11" t="n">
-        <v>8760</v>
+        <v>7350</v>
       </c>
       <c r="G31" s="12" t="n"/>
       <c r="H31">
@@ -3449,6 +3458,12 @@
         <v/>
       </c>
       <c r="J31" s="12" t="n"/>
+      <c r="K31" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="L31" s="11" t="n">
+        <v>21</v>
+      </c>
       <c r="M31" s="12" t="n"/>
       <c r="N31">
         <f>IF(AND(E31="",H31="",J31="",M31=""),"offen",IF(OR(AND(E31&lt;&gt;"",D31&lt;&gt;"",E31&lt;D31),AND(M31&lt;&gt;"",L31&lt;&gt;"",M31&lt;L31)),"unter Alarm",IF(OR(AND(E31&lt;&gt;"",E31&lt;C31),AND(H31&lt;&gt;"",F31&lt;&gt;"",H31&lt;F31),AND(J31&lt;&gt;"",I31&lt;&gt;"",J31&lt;I31),AND(M31&lt;&gt;"",K31&lt;&gt;"",M31&lt;K31)),"unter Soll","im Plan")))</f>
@@ -3456,7 +3471,7 @@
       </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>Do 15.04.: Ware da (spätester Termin)</t>
+          <t>Abi-Pause: keine Gates, Zahlen nur eintragen, wenn du magst</t>
         </is>
       </c>
     </row>
@@ -3470,14 +3485,14 @@
         </is>
       </c>
       <c r="C32" s="11" t="n">
-        <v>3000</v>
+        <v>2450</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>1515</v>
+        <v>880</v>
       </c>
       <c r="E32" s="12" t="n"/>
       <c r="F32" s="11" t="n">
-        <v>9000</v>
+        <v>7350</v>
       </c>
       <c r="G32" s="12" t="n"/>
       <c r="H32">
@@ -3486,10 +3501,10 @@
       </c>
       <c r="J32" s="12" t="n"/>
       <c r="K32" s="11" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="L32" s="11" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="M32" s="12" t="n"/>
       <c r="N32">
@@ -3498,7 +3513,370 @@
       </c>
       <c r="O32" s="3" t="inlineStr">
         <is>
-          <t>Do 22.–So 25.04.: Do 21:00 ≥ 15 · Fr 19:00 ≥ 26 (Schätzung aus Crowdfunding: rund 90 % der Listenkäufer kaufen in 48 h [M-Q27], für Mode nicht belegt) · So ≥ 29 netto</t>
+          <t>Abi-Pause: keine Gates, Zahlen nur eintragen, wenn du magst</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n">
+        <v>46509</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>W33</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>2450</v>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>880</v>
+      </c>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="11" t="n">
+        <v>7350</v>
+      </c>
+      <c r="G33" s="12" t="n"/>
+      <c r="H33">
+        <f>IF(OR(G33="",$C$3=""),"",G33-$C$3)</f>
+        <v/>
+      </c>
+      <c r="J33" s="12" t="n"/>
+      <c r="K33" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="L33" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="M33" s="12" t="n"/>
+      <c r="N33">
+        <f>IF(AND(E33="",H33="",J33="",M33=""),"offen",IF(OR(AND(E33&lt;&gt;"",D33&lt;&gt;"",E33&lt;D33),AND(M33&lt;&gt;"",L33&lt;&gt;"",M33&lt;L33)),"unter Alarm",IF(OR(AND(E33&lt;&gt;"",E33&lt;C33),AND(H33&lt;&gt;"",F33&lt;&gt;"",H33&lt;F33),AND(J33&lt;&gt;"",I33&lt;&gt;"",J33&lt;I33),AND(M33&lt;&gt;"",K33&lt;&gt;"",M33&lt;K33)),"unter Soll","im Plan")))</f>
+        <v/>
+      </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>Abi-Pause: keine Gates, Zahlen nur eintragen, wenn du magst</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n">
+        <v>46516</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>W34</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>2450</v>
+      </c>
+      <c r="D34" s="11" t="n">
+        <v>880</v>
+      </c>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="11" t="n">
+        <v>7350</v>
+      </c>
+      <c r="G34" s="12" t="n"/>
+      <c r="H34">
+        <f>IF(OR(G34="",$C$3=""),"",G34-$C$3)</f>
+        <v/>
+      </c>
+      <c r="J34" s="12" t="n"/>
+      <c r="K34" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="L34" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="M34" s="12" t="n"/>
+      <c r="N34">
+        <f>IF(AND(E34="",H34="",J34="",M34=""),"offen",IF(OR(AND(E34&lt;&gt;"",D34&lt;&gt;"",E34&lt;D34),AND(M34&lt;&gt;"",L34&lt;&gt;"",M34&lt;L34)),"unter Alarm",IF(OR(AND(E34&lt;&gt;"",E34&lt;C34),AND(H34&lt;&gt;"",F34&lt;&gt;"",H34&lt;F34),AND(J34&lt;&gt;"",I34&lt;&gt;"",J34&lt;I34),AND(M34&lt;&gt;"",K34&lt;&gt;"",M34&lt;K34)),"unter Soll","im Plan")))</f>
+        <v/>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>Abi-Pause: keine Gates, Zahlen nur eintragen, wenn du magst</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n">
+        <v>46523</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>W35</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D35" s="11" t="n">
+        <v>910</v>
+      </c>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="11" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35">
+        <f>IF(OR(G35="",$C$3=""),"",G35-$C$3)</f>
+        <v/>
+      </c>
+      <c r="J35" s="12" t="n"/>
+      <c r="K35" s="11" t="n">
+        <v>29</v>
+      </c>
+      <c r="L35" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="M35" s="12" t="n"/>
+      <c r="N35">
+        <f>IF(AND(E35="",H35="",J35="",M35=""),"offen",IF(OR(AND(E35&lt;&gt;"",D35&lt;&gt;"",E35&lt;D35),AND(M35&lt;&gt;"",L35&lt;&gt;"",M35&lt;L35)),"unter Alarm",IF(OR(AND(E35&lt;&gt;"",E35&lt;C35),AND(H35&lt;&gt;"",F35&lt;&gt;"",H35&lt;F35),AND(J35&lt;&gt;"",I35&lt;&gt;"",J35&lt;I35),AND(M35&lt;&gt;"",K35&lt;&gt;"",M35&lt;K35)),"unter Soll","im Plan")))</f>
+        <v/>
+      </c>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t>So 16.05.: ≥ 29 (Alarm 25) · absehbar 32 ausgezahlt bis Di 18.05. (mit der Auszahlungsdauer vom 29.12.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n">
+        <v>46530</v>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>W36</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>2560</v>
+      </c>
+      <c r="D36" s="11" t="n">
+        <v>950</v>
+      </c>
+      <c r="E36" s="12" t="n"/>
+      <c r="F36" s="11" t="n">
+        <v>7680</v>
+      </c>
+      <c r="G36" s="12" t="n"/>
+      <c r="H36">
+        <f>IF(OR(G36="",$C$3=""),"",G36-$C$3)</f>
+        <v/>
+      </c>
+      <c r="J36" s="12" t="n"/>
+      <c r="K36" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="L36" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="M36" s="12" t="n"/>
+      <c r="N36">
+        <f>IF(AND(E36="",H36="",J36="",M36=""),"offen",IF(OR(AND(E36&lt;&gt;"",D36&lt;&gt;"",E36&lt;D36),AND(M36&lt;&gt;"",L36&lt;&gt;"",M36&lt;L36)),"unter Alarm",IF(OR(AND(E36&lt;&gt;"",E36&lt;C36),AND(H36&lt;&gt;"",F36&lt;&gt;"",H36&lt;F36),AND(J36&lt;&gt;"",I36&lt;&gt;"",J36&lt;I36),AND(M36&lt;&gt;"",K36&lt;&gt;"",M36&lt;K36)),"unter Soll","im Plan")))</f>
+        <v/>
+      </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>Fr 21.05.: ≥ 32 ausgezahlt bis Di 18.05. und Endkontroll-Nachweis aus der PO vollständig · So 23.05., 20:00: 35 zu 149 € voll</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="n">
+        <v>46537</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>W37</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>2620</v>
+      </c>
+      <c r="D37" s="11" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="11" t="n">
+        <v>7860</v>
+      </c>
+      <c r="G37" s="12" t="n"/>
+      <c r="H37">
+        <f>IF(OR(G37="",$C$3=""),"",G37-$C$3)</f>
+        <v/>
+      </c>
+      <c r="J37" s="12" t="n"/>
+      <c r="K37" s="11" t="n">
+        <v>37</v>
+      </c>
+      <c r="L37" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="M37" s="12" t="n"/>
+      <c r="N37">
+        <f>IF(AND(E37="",H37="",J37="",M37=""),"offen",IF(OR(AND(E37&lt;&gt;"",D37&lt;&gt;"",E37&lt;D37),AND(M37&lt;&gt;"",L37&lt;&gt;"",M37&lt;L37)),"unter Alarm",IF(OR(AND(E37&lt;&gt;"",E37&lt;C37),AND(H37&lt;&gt;"",F37&lt;&gt;"",H37&lt;F37),AND(J37&lt;&gt;"",I37&lt;&gt;"",J37&lt;I37),AND(M37&lt;&gt;"",K37&lt;&gt;"",M37&lt;K37)),"unter Soll","im Plan")))</f>
+        <v/>
+      </c>
+      <c r="O37" s="3" t="inlineStr">
+        <is>
+          <t>Mi 26.05.: Tracking da · bei Steuer (DAP): 40 ausgezahlt (35 + Stufe 2) · So 30.05.: Ware mit Tracking, Stufe 2 ≥ 2, Kasse deckt die Steuer</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="n">
+        <v>46544</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>W38</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>2720</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>1170</v>
+      </c>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="11" t="n">
+        <v>8160</v>
+      </c>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38">
+        <f>IF(OR(G38="",$C$3=""),"",G38-$C$3)</f>
+        <v/>
+      </c>
+      <c r="J38" s="12" t="n"/>
+      <c r="K38" s="11" t="n">
+        <v>43</v>
+      </c>
+      <c r="M38" s="12" t="n"/>
+      <c r="N38">
+        <f>IF(AND(E38="",H38="",J38="",M38=""),"offen",IF(OR(AND(E38&lt;&gt;"",D38&lt;&gt;"",E38&lt;D38),AND(M38&lt;&gt;"",L38&lt;&gt;"",M38&lt;L38)),"unter Alarm",IF(OR(AND(E38&lt;&gt;"",E38&lt;C38),AND(H38&lt;&gt;"",F38&lt;&gt;"",H38&lt;F38),AND(J38&lt;&gt;"",I38&lt;&gt;"",J38&lt;I38),AND(M38&lt;&gt;"",K38&lt;&gt;"",M38&lt;K38)),"unter Soll","im Plan")))</f>
+        <v/>
+      </c>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>So 06.06.: Ware geprüft, Steuer bezahlt</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="n">
+        <v>46551</v>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>W39</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>2820</v>
+      </c>
+      <c r="D39" s="11" t="n">
+        <v>1290</v>
+      </c>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="11" t="n">
+        <v>8460</v>
+      </c>
+      <c r="G39" s="12" t="n"/>
+      <c r="H39">
+        <f>IF(OR(G39="",$C$3=""),"",G39-$C$3)</f>
+        <v/>
+      </c>
+      <c r="J39" s="12" t="n"/>
+      <c r="M39" s="12" t="n"/>
+      <c r="N39">
+        <f>IF(AND(E39="",H39="",J39="",M39=""),"offen",IF(OR(AND(E39&lt;&gt;"",D39&lt;&gt;"",E39&lt;D39),AND(M39&lt;&gt;"",L39&lt;&gt;"",M39&lt;L39)),"unter Alarm",IF(OR(AND(E39&lt;&gt;"",E39&lt;C39),AND(H39&lt;&gt;"",F39&lt;&gt;"",H39&lt;F39),AND(J39&lt;&gt;"",I39&lt;&gt;"",J39&lt;I39),AND(M39&lt;&gt;"",K39&lt;&gt;"",M39&lt;K39)),"unter Soll","im Plan")))</f>
+        <v/>
+      </c>
+      <c r="O39" s="3" t="inlineStr">
+        <is>
+          <t>Sonntags-Check: Warteliste, Follower, Zusagen bzw. Vorbestellungen gegen das Soll, dazu Kassen-Ampel und Anmeldungen je 1.000 Views (Abschnitt Gates).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="n">
+        <v>46558</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>W40</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="n">
+        <v>2920</v>
+      </c>
+      <c r="D40" s="11" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E40" s="12" t="n"/>
+      <c r="F40" s="11" t="n">
+        <v>8760</v>
+      </c>
+      <c r="G40" s="12" t="n"/>
+      <c r="H40">
+        <f>IF(OR(G40="",$C$3=""),"",G40-$C$3)</f>
+        <v/>
+      </c>
+      <c r="J40" s="12" t="n"/>
+      <c r="M40" s="12" t="n"/>
+      <c r="N40">
+        <f>IF(AND(E40="",H40="",J40="",M40=""),"offen",IF(OR(AND(E40&lt;&gt;"",D40&lt;&gt;"",E40&lt;D40),AND(M40&lt;&gt;"",L40&lt;&gt;"",M40&lt;L40)),"unter Alarm",IF(OR(AND(E40&lt;&gt;"",E40&lt;C40),AND(H40&lt;&gt;"",F40&lt;&gt;"",H40&lt;F40),AND(J40&lt;&gt;"",I40&lt;&gt;"",J40&lt;I40),AND(M40&lt;&gt;"",K40&lt;&gt;"",M40&lt;K40)),"unter Soll","im Plan")))</f>
+        <v/>
+      </c>
+      <c r="O40" s="3" t="inlineStr">
+        <is>
+          <t>Do 17.06.: Ware da (spätester Termin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="n">
+        <v>46565</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>W41</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D41" s="11" t="n">
+        <v>1515</v>
+      </c>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="11" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G41" s="12" t="n"/>
+      <c r="H41">
+        <f>IF(OR(G41="",$C$3=""),"",G41-$C$3)</f>
+        <v/>
+      </c>
+      <c r="J41" s="12" t="n"/>
+      <c r="K41" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="L41" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="M41" s="12" t="n"/>
+      <c r="N41">
+        <f>IF(AND(E41="",H41="",J41="",M41=""),"offen",IF(OR(AND(E41&lt;&gt;"",D41&lt;&gt;"",E41&lt;D41),AND(M41&lt;&gt;"",L41&lt;&gt;"",M41&lt;L41)),"unter Alarm",IF(OR(AND(E41&lt;&gt;"",E41&lt;C41),AND(H41&lt;&gt;"",F41&lt;&gt;"",H41&lt;F41),AND(J41&lt;&gt;"",I41&lt;&gt;"",J41&lt;I41),AND(M41&lt;&gt;"",K41&lt;&gt;"",M41&lt;K41)),"unter Soll","im Plan")))</f>
+        <v/>
+      </c>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>Do 22.–So 27.06.: Do 21:00 ≥ 15 · Fr 19:00 ≥ 26 (Schätzung aus Crowdfunding: rund 90 % der Listenkäufer kaufen in 48 h [M-Q27], für Mode nicht belegt) · So ≥ 29 netto</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3884,7 @@
   <mergeCells count="1">
     <mergeCell ref="A3:B3"/>
   </mergeCells>
-  <conditionalFormatting sqref="N5:N32">
+  <conditionalFormatting sqref="N5:N41">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N5="im Plan"</formula>
     </cfRule>
@@ -3624,7 +4002,7 @@
   </sheetData>
   <dataValidations count="8">
     <dataValidation sqref="A4:A400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Papiertest 24.10.,Stick 27.11.,Creator-Preview 12.01.,Mess 1 16.01.,Mess 2 23.01.,Mess 2b 27.01.,Mess 3 13.03.,Drop-Abend 24.04."</formula1>
+      <formula1>"Papiertest 24.10.,Stick 27.11.,Creator-Preview 12.01.,Mess 1 16.01.,Mess 2 30.01.,Mess 2b 03.02.,Mess 3 15.05.,Drop-Abend 26.06."</formula1>
     </dataValidation>
     <dataValidation sqref="E4:E400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ja,nein"</formula1>
@@ -3674,7 +4052,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Shoot · Sa 20.02.</t>
+          <t>Shoot · Sa 06.03.</t>
         </is>
       </c>
     </row>
@@ -5943,7 +6321,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Drop · 22.–25.04.</t>
+          <t>Drop · 24.–27.06.</t>
         </is>
       </c>
     </row>
@@ -5984,7 +6362,7 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Do 22.04. 21:00</t>
+          <t>Do 24.06. 21:00</t>
         </is>
       </c>
       <c r="B4" s="11" t="n">
@@ -5999,7 +6377,7 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Fr 23.04. 19:00</t>
+          <t>Fr 25.06. 19:00</t>
         </is>
       </c>
       <c r="B5" s="11" t="n">
@@ -6014,7 +6392,7 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>So 25.04. netto</t>
+          <t>So 27.06. netto</t>
         </is>
       </c>
       <c r="B6" s="11" t="n">
@@ -6046,7 +6424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6737,8 +7115,206 @@
         <v/>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="10" t="n">
+        <v>46509</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>W33</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13" t="n"/>
+      <c r="E32" s="13" t="n"/>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="14">
+        <f>IF(C32="","",C32-N(E32)-N(F32))</f>
+        <v/>
+      </c>
+      <c r="H32">
+        <f>IF(G32="","",IF(G32&gt;=300,"grün",IF(G32&gt;=0,"gelb","rot")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n">
+        <v>46516</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>W34</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="n"/>
+      <c r="D33" s="13" t="n"/>
+      <c r="E33" s="13" t="n"/>
+      <c r="F33" s="13" t="n"/>
+      <c r="G33" s="14">
+        <f>IF(C33="","",C33-N(E33)-N(F33))</f>
+        <v/>
+      </c>
+      <c r="H33">
+        <f>IF(G33="","",IF(G33&gt;=300,"grün",IF(G33&gt;=0,"gelb","rot")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n">
+        <v>46523</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>W35</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="n"/>
+      <c r="G34" s="14">
+        <f>IF(C34="","",C34-N(E34)-N(F34))</f>
+        <v/>
+      </c>
+      <c r="H34">
+        <f>IF(G34="","",IF(G34&gt;=300,"grün",IF(G34&gt;=0,"gelb","rot")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n">
+        <v>46530</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>W36</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="n"/>
+      <c r="G35" s="14">
+        <f>IF(C35="","",C35-N(E35)-N(F35))</f>
+        <v/>
+      </c>
+      <c r="H35">
+        <f>IF(G35="","",IF(G35&gt;=300,"grün",IF(G35&gt;=0,"gelb","rot")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n">
+        <v>46537</v>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>W37</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="n"/>
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="14">
+        <f>IF(C36="","",C36-N(E36)-N(F36))</f>
+        <v/>
+      </c>
+      <c r="H36">
+        <f>IF(G36="","",IF(G36&gt;=300,"grün",IF(G36&gt;=0,"gelb","rot")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="n">
+        <v>46544</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>W38</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="n"/>
+      <c r="D37" s="13" t="n"/>
+      <c r="E37" s="13" t="n"/>
+      <c r="F37" s="13" t="n"/>
+      <c r="G37" s="14">
+        <f>IF(C37="","",C37-N(E37)-N(F37))</f>
+        <v/>
+      </c>
+      <c r="H37">
+        <f>IF(G37="","",IF(G37&gt;=300,"grün",IF(G37&gt;=0,"gelb","rot")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="n">
+        <v>46551</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>W39</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="n"/>
+      <c r="D38" s="13" t="n"/>
+      <c r="E38" s="13" t="n"/>
+      <c r="F38" s="13" t="n"/>
+      <c r="G38" s="14">
+        <f>IF(C38="","",C38-N(E38)-N(F38))</f>
+        <v/>
+      </c>
+      <c r="H38">
+        <f>IF(G38="","",IF(G38&gt;=300,"grün",IF(G38&gt;=0,"gelb","rot")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="n">
+        <v>46558</v>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>W40</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="n"/>
+      <c r="D39" s="13" t="n"/>
+      <c r="E39" s="13" t="n"/>
+      <c r="F39" s="13" t="n"/>
+      <c r="G39" s="14">
+        <f>IF(C39="","",C39-N(E39)-N(F39))</f>
+        <v/>
+      </c>
+      <c r="H39">
+        <f>IF(G39="","",IF(G39&gt;=300,"grün",IF(G39&gt;=0,"gelb","rot")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="n">
+        <v>46565</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>W41</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="n"/>
+      <c r="D40" s="13" t="n"/>
+      <c r="E40" s="13" t="n"/>
+      <c r="F40" s="13" t="n"/>
+      <c r="G40" s="14">
+        <f>IF(C40="","",C40-N(E40)-N(F40))</f>
+        <v/>
+      </c>
+      <c r="H40">
+        <f>IF(G40="","",IF(G40&gt;=300,"grün",IF(G40&gt;=0,"gelb","rot")))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="H4:H31">
+  <conditionalFormatting sqref="H4:H40">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$H4="grün"</formula>
     </cfRule>
@@ -7035,7 +7611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7112,12 +7688,12 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>So 11.10.</t>
+          <t>Di 13.10.</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Entschieden: Serp gestrichen · Patch D wird die hintere Gürtelschlaufe (nur seitlich genäht und genietet) · Größe B, 76 × 67 mm, 3–5 mm Spiel</t>
+          <t>Entschieden: Drop verschoben auf Do 24.06.2027 (Abitur). Bis Weihnachten wie geplant, Aufholwochen W19 und W22, Abi-Pause 22.03.–09.05.</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -7132,65 +7708,65 @@
           <t>So 11.10.</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Innenbein-Gradierung +1,0 oder +1,5</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>kein eigener Rat, mir fehlen Daten. Die Spec steht auf +1,0; ohne Grund für +1,5 bleibt es dabei</t>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Entschieden: Serp gestrichen · Patch D wird die hintere Gürtelschlaufe (nur seitlich genäht und genietet) · Größe B, 76 × 67 mm, 3–5 mm Spiel</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>erledigt</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>Do 15.10.</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Wie viel Familie in den Content; Teppich für den Shoot leihen</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>über Gegenstände, nicht über Länder</t>
+          <t>So 11.10.</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Innenbein-Gradierung +1,0 oder +1,5</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>kein eigener Rat, mir fehlen Daten. Die Spec steht auf +1,0; ohne Grund für +1,5 bleibt es dabei</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>So 18.10.</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Pixel-Spiel</t>
+          <t>Do 15.10.</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Wie viel Familie in den Content; Teppich für den Shoot leihen</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>streichen, Scroll-Story B</t>
+          <t>über Gegenstände, nicht über Länder</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Di 20.10.</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Patch D: mittig auf der hinteren Mittelnaht oder rechts daneben; „NL“ auf dem Patch</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>mittig, wenn die Fabrik Nieten über der Mittelnaht bestätigt; NL wie auf dem Foto</t>
+          <t>So 18.10.</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Pixel-Spiel</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>streichen, Scroll-Story B</t>
         </is>
       </c>
     </row>
@@ -7202,143 +7778,143 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Baum-Referenz: eigene oder fremde Vorlage?</t>
+          <t>Patch D: mittig auf der hinteren Mittelnaht oder rechts daneben; „NL“ auf dem Patch</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>fremd → Claude zeichnet eine eigene Fassung vor dem 28.10.</t>
+          <t>mittig, wenn die Fabrik Nieten über der Mittelnaht bestätigt; NL wie auf dem Foto</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>ab So 01.11.</t>
+          <t>Di 20.10.</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>IHK-Gründungsberatung (angefragt am 13.10.), danach Gewerbe anmelden</t>
+          <t>Baum-Referenz: eigene oder fremde Vorlage?</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>anmelden vor der ersten Vorbestellung und bevor Rechnungen auf deinen Namen laufen; online geht es in 20 Minuten</t>
+          <t>fremd → Claude zeichnet eine eigene Fassung vor dem 28.10.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Di 27.10.</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>DAP oder DDP</t>
+          <t>ab So 01.11.</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>IHK-Gründungsberatung (angefragt am 13.10.), danach Gewerbe anmelden</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>DAP, damit die Steuer nicht schon in der Restzahlung steckt</t>
+          <t>anmelden vor der ersten Vorbestellung und bevor Rechnungen auf deinen Namen laufen; online geht es in 20 Minuten</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Sa 07.11.</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Sprache der Hooks und damit das Liefergebiet; Bildregel „keine Seitenansicht links“</t>
+          <t>Di 27.10.</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>DAP oder DDP</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Test entscheidet; deutsch → nur Versand nach DE bis zum Drop; Bildregel halten</t>
+          <t>DAP, damit die Steuer nicht schon in der Restzahlung steckt</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>So 29.11.</t>
+          <t>Sa 07.11.</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>„Platz in der ersten Stunde sichern“ A (10 €) oder B (kostenlos)</t>
+          <t>Sprache der Hooks und damit das Liefergebiet; Bildregel „keine Seitenansicht links“</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>B, A nur bei Liste &lt; 170 und grünem Recht</t>
+          <t>Test entscheidet; deutsch → nur Versand nach DE bis zum Drop; Bildregel halten</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Fr 11.12.</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Creator-Abmachung 1 Clip + 1 Story</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>So 29.11.</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>„Platz in der ersten Stunde sichern“ A (10 €) oder B (kostenlos)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>B, A nur bei Liste &lt; 170 und grünem Recht</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Mo 14.12.</t>
+          <t>Fr 11.12.</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Liefertext</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>„Lieferung bis spätestens 30.04.2027, geplant Anfang April“, überall derselbe Satz</t>
+          <t>Creator-Abmachung 1 Clip + 1 Story</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>ja</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Di 15.12.</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Geld-zurück-Regel, Vorbestellgeld bis 01.02. unangetastet</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>ja</t>
+          <t>Mo 14.12.</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Liefertext</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>„Lieferung bis spätestens 30.06.2027, geplant Anfang Juni“, überall derselbe Satz</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Sa 19.12.</t>
+          <t>Di 15.12.</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Stufe 2 zu 169 € statt Kontingent 45; Nummern 001–035 · 036–060 · 061–065 · 066–067 · Rest</t>
+          <t>Geld-zurück-Regel, Vorbestellgeld bis 15.02. unangetastet</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -7350,83 +7926,100 @@
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Do 31.12.</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Brücke 1.500 € in der Familie</t>
+          <t>Sa 19.12.</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Stufe 2 zu 169 € statt Kontingent 45; Nummern 001–035 · 036–060 · 061–065 · 066–067 · Rest</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>anfragen, nur als Versicherung</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>So 24.01.</t>
+          <t>Do 31.12.</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Mess-Abend 2b (Mi 27.01.)</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>ja, wenn am 13.01. &lt; 60 Reservierungen + Zusagen oder Vorbestellungen unter Soll</t>
+          <t>Brücke 1.500 € in der Familie</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>anfragen, nur als Versicherung</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Mo 01.02.</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Mengenformel 100/75; Notfall-Option Zipper bei 7–9</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>ja / bereithalten</t>
+          <t>So 31.01.</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Mess-Abend 2b (Mi 03.02.)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>ja, wenn am 13.01. &lt; 60 Reservierungen + Zusagen oder Vorbestellungen unter Soll</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Fr 05.03.</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Drop-Abend Sa 24.04.; Countdown-Stand</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>ja nur, wenn Packen Tag 2 an die Helfer geht oder auf So 25.04. rückt / nur unter ~146 €</t>
+          <t>Mo 15.02.</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Mengenformel 100/75; Notfall-Option Zipper bei 7–9</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>ja / bereithalten</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
+          <t>Fr 19.03.</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Drop-Abend Sa 26.06.; Countdown-Stand</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>ja nur, wenn Packen Tag 2 an die Helfer geht oder auf So 27.06. rückt / nur unter ~146 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
           <t>nach dem Drop</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Marke „Novalife“ anmelden; W28 in den Größenlauf</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Markenrecherche vom 16.10. und Nachfrage „kleiner als W30“ auswerten, erst dann rechnen</t>
         </is>
@@ -8043,7 +8636,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>bei Einfuhr ~25.–30.03.</t>
+          <t>bei Einfuhr ~27.05.–01.06.</t>
         </is>
       </c>
       <c r="E24" s="16" t="n"/>
@@ -8746,7 +9339,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>zweites Proto, Öffnung nach B-Zeitachse 1 (Do 21.01.)</t>
+          <t>zweites Proto, Öffnung nach B-Zeitachse 1 (Do 28.01.)</t>
         </is>
       </c>
     </row>
@@ -8790,7 +9383,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>&lt; 10 Zusagen: Ausgaben-Stopp, Proto-Runde verlängern · Auszahlung unklar: kein Start · Patch offen: Bestellung Mo 21.12., Fabrik über neue Patch-Frist Fr 29.01. informieren</t>
+          <t>&lt; 10 Zusagen: Ausgaben-Stopp, Proto-Runde verlängern · Auszahlung unklar: kein Start · Patch offen: Bestellung Mo 21.12., Fabrik über neue Patch-Frist Fr 05.02. informieren</t>
         </is>
       </c>
     </row>
@@ -8812,7 +9405,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Öffnung höchstens Do 21.01. (B-Zeitachse 1)</t>
+          <t>Öffnung höchstens Do 28.01. (B-Zeitachse 1)</t>
         </is>
       </c>
     </row>
@@ -8863,7 +9456,7 @@
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>So 24.01.</t>
+          <t>So 31.01.</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -8878,24 +9471,24 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>1,0–1,5 %: Mess-Abend 13.03. als Hauptereignis · &lt; 1,0 %: Grind+-Ziel 3.390 wird Pflicht · Mess-Abend 2b am Mi 27.01. (Do 28.01. nur bei Auszahlung ≤ 2 Werktage), wenn am 13.01. &lt; 60 Reservierungen + Zusagen oder Vorbestellungen unter Soll · Patches fehlen: Call und neue Rechnung für den Produktionsstart</t>
+          <t>1,0–1,5 %: Mess-Abend 15.05. als Hauptereignis · &lt; 1,0 %: Grind+-Ziel 3.390 wird Pflicht · Mess-Abend 2b am Mi 03.02. (Do 04.02. nur bei Auszahlung ≤ 2 Werktage), wenn am 13.01. &lt; 60 Reservierungen + Zusagen oder Vorbestellungen unter Soll · Patches fehlen: Call und neue Rechnung für den Produktionsstart</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Mo 01.02.</t>
+          <t>Mo 15.02.</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Schwelle 1 + Mengenformel (ausgezahlt am 31.01. + 6 × Wochenrate W19–W20)</t>
+          <t>Schwelle 1 + Mengenformel (ausgezahlt am 07.02. + 6 × Wochenrate W19–W20)</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>≥ 10 und Hochrechnung ≥ 32 ausgezahlt bis Di 16.03. → 100 Stück (bei Steuer zusätzlich 40 bis Mi 24.03. inkl. Stufe 2)</t>
+          <t>≥ 10 und Hochrechnung ≥ 32 ausgezahlt bis Di 18.05. → 100 Stück (bei Steuer zusätzlich 40 bis Mi 26.05. inkl. Stufe 2)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -8907,7 +9500,7 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Fr 05.02.</t>
+          <t>Fr 19.02.</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
@@ -8929,7 +9522,7 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>So 07.02.</t>
+          <t>So 21.02.</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -8951,7 +9544,7 @@
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>So 14.02.</t>
+          <t>So 28.02.</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
@@ -8973,7 +9566,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>So 21.02.</t>
+          <t>So 07.03.</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -8995,7 +9588,7 @@
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>So 28.02.</t>
+          <t>So 14.03.</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -9017,7 +9610,7 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>So 07.03.</t>
+          <t>So 21.03.</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -9039,34 +9632,34 @@
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>So 14.03.</t>
+          <t>So 16.05.</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>≥ 29 (Alarm 25) · absehbar 32 ausgezahlt bis Di 16.03. (mit der Auszahlungsdauer vom 29.12.)</t>
+          <t>≥ 29 (Alarm 25) · absehbar 32 ausgezahlt bis Di 18.05. (mit der Auszahlungsdauer vom 29.12.)</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Restzahlung 19.03.</t>
+          <t>Restzahlung 21.05.</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Notfall-Leiter ab Stufe 3, Backstop Mi 24.03. vorbereiten</t>
+          <t>Notfall-Leiter ab Stufe 3, Backstop Mi 26.05. vorbereiten</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Fr 19.03.</t>
+          <t>Fr 21.05.</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>≥ 32 ausgezahlt bis Di 16.03. und Endkontroll-Nachweis aus der PO vollständig</t>
+          <t>≥ 32 ausgezahlt bis Di 18.05. und Endkontroll-Nachweis aus der PO vollständig</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -9076,14 +9669,14 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>nur Geld fehlt: Backstop Mi 24.03. · Endkontrolle durchgefallen: nicht zahlen, Fotos an die Fabrik</t>
+          <t>nur Geld fehlt: Backstop Mi 26.05. · Endkontrolle durchgefallen: nicht zahlen, Fotos an die Fabrik</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>So 21.03., 20:00</t>
+          <t>So 23.05., 20:00</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
@@ -9098,14 +9691,14 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>149 € endet trotzdem; Stufe 2 läuft spätestens ab jetzt bis So 04.04. Preis nie verlängern</t>
+          <t>149 € endet trotzdem; Stufe 2 läuft spätestens ab jetzt bis So 06.06. Preis nie verlängern</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Mi 24.03.</t>
+          <t>Mi 26.05.</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -9120,14 +9713,14 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>tägliche Mail an die Fabrik, ab 31.03. Drop-Plan B · Steuer-Geld fehlt: Brücke abrufen (Stufe 7)</t>
+          <t>tägliche Mail an die Fabrik, ab 02.06. Drop-Plan B · Steuer-Geld fehlt: Brücke abrufen (Stufe 7)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>So 28.03.</t>
+          <t>So 30.05.</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -9142,14 +9735,14 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Stufe 2 &lt; 2: Mail und Story „Stufe 2 bis 04.04.“ · Steuer nicht gedeckt: Brücke abrufen</t>
+          <t>Stufe 2 &lt; 2: Mail und Story „Stufe 2 bis 06.06.“ · Steuer nicht gedeckt: Brücke abrufen</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>So 04.04.</t>
+          <t>So 06.06.</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -9171,7 +9764,7 @@
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>Do 15.04.</t>
+          <t>Do 17.06.</t>
         </is>
       </c>
       <c r="B37" s="11" t="inlineStr">
@@ -9181,19 +9774,19 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Drop 22.04.</t>
+          <t>Drop 24.06.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Drop 29.04. (B-Zeitachse 2) oder „Versand ab Ankunft“, offen angekündigt [P 6] · Ware erst nach So 25.04.: Mail an alle Vorbesteller mit neuem Datum und dem Angebot voller Erstattung</t>
+          <t>Drop 01.07. (B-Zeitachse 2) oder „Versand ab Ankunft“, offen angekündigt [P 6] · Ware erst nach So 27.06.: Mail an alle Vorbesteller mit neuem Datum und dem Angebot voller Erstattung</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>Do 22.–So 25.04.</t>
+          <t>Do 24.–So 27.06.</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">

</xml_diff>